<commit_message>
modified the data import part, it now pulls the factor levels already present in the experiment and then runs the import factor using the miappe template ONLY if it stumbles on an unkown factor level. If the facor level is valid and created by this, it can continue to run, if not, the program stops.
</commit_message>
<xml_diff>
--- a/exp_database/test_JACOS/RGB1_Morpho_Manual.xlsx
+++ b/exp_database/test_JACOS/RGB1_Morpho_Manual.xlsx
@@ -308,87 +308,87 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -651,19 +651,19 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="4" width="20.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="5" width="10.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="4" width="11.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="4" width="11.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="4" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="5" width="9.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="3" width="9.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="3" width="15.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="3" width="9.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="6" width="10.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="6" width="10.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="6" width="14.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="6" width="16.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="6" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="3" width="10.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="3" width="10.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="6" width="12.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="3" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="6" width="12.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="6" width="12.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="4" width="13.01"/>
   </cols>
   <sheetData>

</xml_diff>